<commit_message>
update: Shioaji 实时行情同步 [2026-08-20 13:15:06] (v20260820_131506)
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-08-12 13:35:51 | 数据源: 永丰金 Shioaji API (TWSE 实时盘口) | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-08-20 13:14:56 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -730,10 +730,10 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>开盘: 2405.0
-最高: 2415.0
-最低: 2390.0
-收盘: 2415.0</t>
+          <t>开盘: 2365.0
+最高: 2370.0
+最低: 2350.0
+收盘: 2365.0</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2415.0</t>
+          <t>NT$ 2365.0</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>17,595 张</t>
+          <t>10,000 张</t>
         </is>
       </c>
     </row>
@@ -817,10 +817,10 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>开盘: 12250.0
-最高: 12295.0
-最低: 11790.0
-收盘: 12045.0</t>
+          <t>开盘: 14245.0
+最高: 14495.0
+最低: 13795.0
+收盘: 14080.0</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 12045.0</t>
+          <t>NT$ 14080.0</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="O5" s="16" t="inlineStr">
         <is>
-          <t>309 张</t>
+          <t>470 张</t>
         </is>
       </c>
     </row>
@@ -904,10 +904,10 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>开盘: 5500.0
-最高: 5730.0
-最低: 5480.0
-收盘: 5730.0</t>
+          <t>开盘: 6100.0
+最高: 6200.0
+最低: 5780.0
+收盘: 5960.0</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5730.0</t>
+          <t>NT$ 5960.0</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>1,464 张</t>
+          <t>2,164 张</t>
         </is>
       </c>
     </row>
@@ -991,10 +991,10 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>开盘: 2765.0
-最高: 2915.0
-最低: 2755.0
-收盘: 2910.0</t>
+          <t>开盘: 3175.0
+最高: 3175.0
+最低: 2925.0
+收盘: 2960.0</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2910.0</t>
+          <t>NT$ 2960.0</t>
         </is>
       </c>
       <c r="K7" s="18" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>3,888 张</t>
+          <t>2,535 张</t>
         </is>
       </c>
     </row>
@@ -1078,10 +1078,10 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>开盘: 264.5
-最高: 270.5
-最低: 264.0
-收盘: 270.0</t>
+          <t>开盘: 250.5
+最高: 250.5
+最低: 244.0
+收盘: 245.5</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 270.0</t>
+          <t>NT$ 245.5</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>57,458 张</t>
+          <t>20,676 张</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-08-12 13:35:51 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-08-20 13:14:56 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>
@@ -1250,22 +1250,22 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2405.0</t>
+          <t>NT$ 2365.0</t>
         </is>
       </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2415.0</t>
+          <t>NT$ 2370.0</t>
         </is>
       </c>
       <c r="E4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2390.0</t>
+          <t>NT$ 2350.0</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2415.0</t>
+          <t>NT$ 2365.0</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
@@ -1297,22 +1297,22 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 12250.0</t>
+          <t>NT$ 14245.0</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 12295.0</t>
+          <t>NT$ 14495.0</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 11790.0</t>
+          <t>NT$ 13795.0</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 12045.0</t>
+          <t>NT$ 14080.0</t>
         </is>
       </c>
       <c r="G5" s="29" t="inlineStr">
@@ -1344,22 +1344,22 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5500.0</t>
+          <t>NT$ 6100.0</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5730.0</t>
+          <t>NT$ 6200.0</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5480.0</t>
+          <t>NT$ 5780.0</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5730.0</t>
+          <t>NT$ 5960.0</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
@@ -1391,22 +1391,22 @@
       </c>
       <c r="C7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2765.0</t>
+          <t>NT$ 3175.0</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2915.0</t>
+          <t>NT$ 3175.0</t>
         </is>
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2755.0</t>
+          <t>NT$ 2925.0</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2910.0</t>
+          <t>NT$ 2960.0</t>
         </is>
       </c>
       <c r="G7" s="29" t="inlineStr">
@@ -1438,22 +1438,22 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 264.5</t>
+          <t>NT$ 250.5</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 270.5</t>
+          <t>NT$ 250.5</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 264.0</t>
+          <t>NT$ 244.0</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 270.0</t>
+          <t>NT$ 245.5</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">

</xml_diff>

<commit_message>
update: Shioaji 实时行情同步 [2026-08-21 22:08:14] (v20260821_220814)
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-08-20 13:14:56 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-08-21 22:08:14 | 数据源: Shioaji Snapshot | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -730,10 +730,10 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>开盘: 2365.0
-最高: 2370.0
-最低: 2350.0
-收盘: 2365.0</t>
+          <t>开盘: 2375.0
+最高: 2410.0
+最低: 2365.0
+收盘: 2410.0</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -751,15 +751,15 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>外资: +2,450 张
-投信: +680 张
-外资持股 74.2%，高档回调接盘，投信连续 5 日买超，主力资金控盘极稳。</t>
+          <t>外资: +5795 张
+投信: +291 张
+[2026-08-21 官方结算] 三大法人全线买超 (+6,543 张)，外资与投信合力加仓。</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>62.5% 买盘大单
-主力资金呈净流入 (+18.5 亿 NTD)，散户筹码清洗彻底。</t>
+          <t>法人净买超 6,543 张 (占量 41.6%)
+[2026-08-21 筹码] 主力机构呈净买入 (+6,543 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2365.0</t>
+          <t>NT$ 2410.0</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>10,000 张</t>
+          <t>15,735 张</t>
         </is>
       </c>
     </row>
@@ -817,10 +817,10 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>开盘: 14245.0
-最高: 14495.0
-最低: 13795.0
-收盘: 14080.0</t>
+          <t>开盘: 13900.0
+最高: 14000.0
+最低: 13310.0
+收盘: 13385.0</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -838,15 +838,15 @@
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>外资: -15 张
-投信: +120 张
-内资投信死锁筹码，外资高档极少调节，筹码集中度高达 82%。</t>
+          <t>外资: +37 张
+投信: +25 张
+[2026-08-21 官方结算] 三大法人全线买超 (+69 张)，外资与投信合力加仓。</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>71.0% 法人特定大单
-高单价低流动性，主力锁筹意愿极强，空头无借券源（易轧空）。</t>
+          <t>法人净买超 69 张 (占量 11.5%)
+[2026-08-21 筹码] 主力机构呈净买入 (+69 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I5" s="15" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 14080.0</t>
+          <t>NT$ 13385.0</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="O5" s="16" t="inlineStr">
         <is>
-          <t>470 张</t>
+          <t>602 张</t>
         </is>
       </c>
     </row>
@@ -904,10 +904,10 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>开盘: 6100.0
-最高: 6200.0
-最低: 5780.0
-收盘: 5960.0</t>
+          <t>开盘: 6005.0
+最高: 6015.0
+最低: 5650.0
+收盘: 5680.0</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -925,15 +925,15 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>外资: +850 张
-投信: +1,120 张
-三大法人同步买超（买超最强），主力资金连续 8 日流入。</t>
+          <t>外资: +379 张
+投信: -410 张
+[2026-08-21 官方结算] 外资主力大幅回流 (+379 张)，投信阶段获利减仓 (-410 张)。</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>68.4% 主力大单
-M8/M9 材料放量带起涨价潮，资金流入显著加快。</t>
+          <t>法人净买超 49 张 (占量 2.3%)
+[2026-08-21 筹码] 主力机构呈净买入 (+49 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5960.0</t>
+          <t>NT$ 5680.0</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>2,164 张</t>
+          <t>2,132 张</t>
         </is>
       </c>
     </row>
@@ -991,10 +991,10 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>开盘: 3175.0
-最高: 3175.0
-最低: 2925.0
-收盘: 2960.0</t>
+          <t>开盘: 2995.0
+最高: 3035.0
+最低: 2850.0
+收盘: 2865.0</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -1012,15 +1012,15 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>外资: -320 张
-投信: +1,450 张
-外资洗盘抛售，但投信逢低狂吞大吃，投信呈现单边净买超。</t>
+          <t>外资: -68 张
+投信: +44 张
+[2026-08-21 官方结算] 投信内资买超 (+44 张) 逢低承接，外资高档调节 (-68 张)。</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>59.2% 大单比重
-水冷良率及出货背书，内资主力坚定接盘。</t>
+          <t>法人净卖超 80 张 (占量 3.5%)
+[2026-08-21 筹码] 主力机构呈净卖出 (-80 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2960.0</t>
+          <t>NT$ 2865.0</t>
         </is>
       </c>
       <c r="K7" s="18" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>2,535 张</t>
+          <t>2,309 张</t>
         </is>
       </c>
     </row>
@@ -1078,9 +1078,9 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>开盘: 250.5
-最高: 250.5
-最低: 244.0
+          <t>开盘: 245.0
+最高: 247.0
+最低: 243.0
 收盘: 245.5</t>
         </is>
       </c>
@@ -1099,15 +1099,15 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>外资: +12,400 张
-投信: +2,100 张
-三大法人全线买超 (+1.63 万张)，外资巨量买盘回流第一名。</t>
+          <t>外资: -3529 张
+投信: +66 张
+[2026-08-21 官方结算] 投信内资买超 (+66 张) 逢低承接，外资高档调节 (-3,529 张)。</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>74.8% 机构级买单
-巨额资金持续流入，AI 伺服器占比突破 50% 引发重估潮。</t>
+          <t>法人净卖超 3,376 张 (占量 14.0%)
+[2026-08-21 筹码] 主力机构呈净卖出 (-3,376 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>20,676 张</t>
+          <t>24,136 张</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-08-20 13:14:56 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-08-21 22:08:14 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>
@@ -1250,22 +1250,22 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
+          <t>NT$ 2375.0</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 2410.0</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
           <t>NT$ 2365.0</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
-        <is>
-          <t>NT$ 2370.0</t>
-        </is>
-      </c>
-      <c r="E4" s="24" t="inlineStr">
-        <is>
-          <t>NT$ 2350.0</t>
-        </is>
-      </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2365.0</t>
+          <t>NT$ 2410.0</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
@@ -1297,22 +1297,22 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 14245.0</t>
+          <t>NT$ 13900.0</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 14495.0</t>
+          <t>NT$ 14000.0</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 13795.0</t>
+          <t>NT$ 13310.0</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 14080.0</t>
+          <t>NT$ 13385.0</t>
         </is>
       </c>
       <c r="G5" s="29" t="inlineStr">
@@ -1344,22 +1344,22 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6100.0</t>
+          <t>NT$ 6005.0</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6200.0</t>
+          <t>NT$ 6015.0</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5780.0</t>
+          <t>NT$ 5650.0</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5960.0</t>
+          <t>NT$ 5680.0</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
@@ -1391,22 +1391,22 @@
       </c>
       <c r="C7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3175.0</t>
+          <t>NT$ 2995.0</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3175.0</t>
+          <t>NT$ 3035.0</t>
         </is>
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2925.0</t>
+          <t>NT$ 2850.0</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2960.0</t>
+          <t>NT$ 2865.0</t>
         </is>
       </c>
       <c r="G7" s="29" t="inlineStr">
@@ -1438,17 +1438,17 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 250.5</t>
+          <t>NT$ 245.0</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 250.5</t>
+          <t>NT$ 247.0</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 244.0</t>
+          <t>NT$ 243.0</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">

</xml_diff>

<commit_message>
data: publish ten-stock quote payload
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -624,14 +624,14 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表</t>
+          <t>台股 10 檔 AI 核心卡位龙头深度投资与买卖点筹码量化分析表</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-08-26 15:24:17 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-08-27 16:29:12 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -730,10 +730,10 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>开盘: 2375.0
-最高: 2425.0
-最低: 2375.0
-收盘: 2415.0</t>
+          <t>开盘: 2430.0
+最高: 2435.0
+最低: 2410.0
+收盘: 2410.0</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -751,15 +751,15 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>外资: +2,450 张
-投信: +680 张
-外资持股 74.2%，高档回调接盘，投信连续 5 日买超，主力资金控盘极稳。</t>
+          <t>外资: +5204 张
+投信: -521 张
+[2026-08-26 官方结算] 外资主力大幅回流 (+5,204 张)，投信阶段获利减仓 (-521 张)。</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>62.5% 买盘大单
-主力资金呈净流入 (+18.5 亿 NTD)，散户筹码清洗彻底。</t>
+          <t>法人净买超 4,910 张 (占量 30.3%)
+[2026-08-26 筹码] 主力机构呈净买入 (+4,910 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2415.0</t>
+          <t>NT$ 2410.0</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>17,627 张</t>
+          <t>16,222 张</t>
         </is>
       </c>
     </row>
@@ -817,10 +817,10 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>开盘: 14295.0
-最高: 14590.0
-最低: 13855.0
-收盘: 14510.0</t>
+          <t>开盘: 14695.0
+最高: 14815.0
+最低: 14085.0
+收盘: 14340.0</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -838,15 +838,15 @@
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>外资: -15 张
-投信: +120 张
-内资投信死锁筹码，外资高档极少调节，筹码集中度高达 82%。</t>
+          <t>外资: +43 张
+投信: -9 张
+[2026-08-26 官方结算] 外资主力大幅回流 (+43 张)，投信阶段获利减仓 (-9 张)。</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>71.0% 法人特定大单
-高单价低流动性，主力锁筹意愿极强，空头无借券源（易轧空）。</t>
+          <t>法人净买超 56 张 (占量 16.3%)
+[2026-08-26 筹码] 主力机构呈净买入 (+56 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I5" s="15" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 14510.0</t>
+          <t>NT$ 14340.0</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="O5" s="16" t="inlineStr">
         <is>
-          <t>463 张</t>
+          <t>343 张</t>
         </is>
       </c>
     </row>
@@ -904,10 +904,10 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>开盘: 5565.0
-最高: 5920.0
-最低: 5555.0
-收盘: 5895.0</t>
+          <t>开盘: 5960.0
+最高: 5960.0
+最低: 5355.0
+收盘: 5500.0</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -925,15 +925,15 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>外资: +850 张
-投信: +1,120 张
-三大法人同步买超（买超最强），主力资金连续 8 日流入。</t>
+          <t>外资: +52 张
+投信: +43 张
+[2026-08-26 官方结算] 外资与投信联手买超 (+75 张)，内外部机构共振做多。</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>68.4% 主力大单
-M8/M9 材料放量带起涨价潮，资金流入显著加快。</t>
+          <t>法人净买超 75 张 (占量 2.4%)
+[2026-08-26 筹码] 主力机构呈净买入 (+75 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5895.0</t>
+          <t>NT$ 5500.0</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>1,752 张</t>
+          <t>3,079 张</t>
         </is>
       </c>
     </row>
@@ -991,10 +991,10 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>开盘: 2880.0
-最高: 3155.0
-最低: 2850.0
-收盘: 3155.0</t>
+          <t>开盘: 3305.0
+最高: 3440.0
+最低: 3265.0
+收盘: 3340.0</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -1012,15 +1012,15 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>外资: -320 张
-投信: +1,450 张
-外资洗盘抛售，但投信逢低狂吞大吃，投信呈现单边净买超。</t>
+          <t>外资: -623 张
+投信: +440 张
+[2026-08-26 官方结算] 投信内资买超 (+440 张) 逢低承接，外资高档调节 (-623 张)。</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>59.2% 大单比重
-水冷良率及出货背书，内资主力坚定接盘。</t>
+          <t>法人净卖超 62 张 (占量 1.1%)
+[2026-08-26 筹码] 主力机构呈净卖出 (-62 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3155.0</t>
+          <t>NT$ 3340.0</t>
         </is>
       </c>
       <c r="K7" s="18" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>4,944 张</t>
+          <t>5,609 张</t>
         </is>
       </c>
     </row>
@@ -1078,10 +1078,10 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>开盘: 243.0
-最高: 248.0
-最低: 241.5
-收盘: 246.5</t>
+          <t>开盘: 248.5
+最高: 256.5
+最低: 248.5
+收盘: 252.0</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1099,15 +1099,15 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>外资: +12,400 张
-投信: +2,100 张
-三大法人全线买超 (+1.63 万张)，外资巨量买盘回流第一名。</t>
+          <t>外资: -2072 张
+投信: +11 张
+[2026-08-26 官方结算] 投信内资买超 (+11 张) 逢低承接，外资高档调节 (-2,072 张)。</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>74.8% 机构级买单
-巨额资金持续流入，AI 伺服器占比突破 50% 引发重估潮。</t>
+          <t>法人净卖超 1,358 张 (占量 3.3%)
+[2026-08-26 筹码] 主力机构呈净卖出 (-1,358 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 246.5</t>
+          <t>NT$ 252.0</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
@@ -1143,7 +1143,442 @@
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>23,519 张</t>
+          <t>40,735 张</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="105" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>2308.TW</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>台達電</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>高效率電源、資料中心基礎設施與熱管理的系統級整合</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>开盘: 1780.0
+最高: 1820.0
+最低: 1760.0
+收盘: 1770.0</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>• 毛利率：35.6% (26Q2)
+• 净利率：13.7% (26Q2)
+• ROE：待更新
+• EPS：9.68 元 (26Q2)</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>2026Q2 已公告；下一次財報/法說日待公司公告</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>外资: +605 张
+投信: -1707 张
+[2026-08-26 官方结算] 外资主力大幅回流 (+605 张)，投信阶段获利减仓 (-1,707 张)。</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>法人净卖超 860 张 (占量 10.4%)
+[2026-08-26 筹码] 主力机构呈净卖出 (-860 张)，散户承接，筹码短期发散。</t>
+        </is>
+      </c>
+      <c r="I9" s="15" t="inlineStr">
+        <is>
+          <t>【Chokepoint 85分】卡位最上游铲子卖家，客户切换周期超 12-36 个月，垄断护城河极深。</t>
+        </is>
+      </c>
+      <c r="J9" s="17" t="inlineStr">
+        <is>
+          <t>NT$ 1770.0</t>
+        </is>
+      </c>
+      <c r="K9" s="18" t="inlineStr">
+        <is>
+          <t>建议买点：分批觀察（不追高）
+黄金重仓：等待估值明顯回落</t>
+        </is>
+      </c>
+      <c r="L9" s="19" t="inlineStr">
+        <is>
+          <t>依獲利與趨勢再評估</t>
+        </is>
+      </c>
+      <c r="M9" s="20" t="inlineStr">
+        <is>
+          <t>不預設固定目標</t>
+        </is>
+      </c>
+      <c r="N9" s="21" t="inlineStr">
+        <is>
+          <t>跌破基本面假設即檢視</t>
+        </is>
+      </c>
+      <c r="O9" s="16" t="inlineStr">
+        <is>
+          <t>8,286 张</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="105" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2345.TW</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>智邦</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>800G/1.6T 高速交換器與 AI 集群網路整合的高門檻環節</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>开盘: 2120.0
+最高: 2130.0
+最低: 2065.0
+收盘: 2090.0</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>• 毛利率：19.7% (26Q2)
+• 净利率：約 11.6% (26Q2)
+• ROE：待更新
+• EPS：19.78 元 (26Q2)</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>2026Q2 已公告；下一次財報/法說日待公司公告</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>外资: +325 张
+投信: -617 张
+[2026-08-26 官方结算] 外资主力大幅回流 (+325 张)，投信阶段获利减仓 (-617 张)。</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>法人净卖超 262 张 (占量 11.1%)
+[2026-08-26 筹码] 主力机构呈净卖出 (-262 张)，散户承接，筹码短期发散。</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>【Chokepoint 86分】卡位最上游铲子卖家，客户切换周期超 12-36 个月，垄断护城河极深。</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>NT$ 2090.0</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>建议买点：分批觀察（不追高）
+黄金重仓：等待成長預期降溫</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>依訂單與 EPS 趨勢再評估</t>
+        </is>
+      </c>
+      <c r="M10" s="11" t="inlineStr">
+        <is>
+          <t>不預設固定目標</t>
+        </is>
+      </c>
+      <c r="N10" s="12" t="inlineStr">
+        <is>
+          <t>營益率與訂單能見度轉弱即檢視</t>
+        </is>
+      </c>
+      <c r="O10" s="7" t="inlineStr">
+        <is>
+          <t>2,370 张</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="105" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>2360.TW</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>致茂</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>高精度測試、量測與先進封裝檢測，屬 AI 硬體量產的關鍵驗證設備</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>开盘: 2010.0
+最高: 2085.0
+最低: 1970.0
+收盘: 1990.0</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>• 毛利率：約 60.5% (26Q2)
+• 净利率：約 37.9% (26Q2)
+• ROE：待更新
+• EPS：約 12.15 元 (26Q2)</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>2026Q2 已公告；下一次財報/法說日待公司公告</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>外资: -186 张
+投信: -131 张
+[2026-08-26 官方结算] 外资与投信偏空调节 (-242 张)，机构筹码阶段获利了结。</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>法人净卖超 242 张 (占量 13.4%)
+[2026-08-26 筹码] 主力机构呈净卖出 (-242 张)，散户承接，筹码短期发散。</t>
+        </is>
+      </c>
+      <c r="I11" s="15" t="inlineStr">
+        <is>
+          <t>【Chokepoint 84分】卡位最上游铲子卖家，客户切换周期超 12-36 个月，垄断护城河极深。</t>
+        </is>
+      </c>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>NT$ 1990.0</t>
+        </is>
+      </c>
+      <c r="K11" s="18" t="inlineStr">
+        <is>
+          <t>建议买点：回檔分批觀察
+黄金重仓：等待估值與波動收斂</t>
+        </is>
+      </c>
+      <c r="L11" s="19" t="inlineStr">
+        <is>
+          <t>依 EPS 與毛利率再評估</t>
+        </is>
+      </c>
+      <c r="M11" s="20" t="inlineStr">
+        <is>
+          <t>不預設固定目標</t>
+        </is>
+      </c>
+      <c r="N11" s="21" t="inlineStr">
+        <is>
+          <t>獲利趨勢反轉即檢視</t>
+        </is>
+      </c>
+      <c r="O11" s="16" t="inlineStr">
+        <is>
+          <t>1,800 张</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="105" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>3711.TW</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>日月光投控</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>AI 晶片大規模封裝測試與先進封裝產能，屬量產環節的關鍵瓶頸</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>开盘: 608.0
+最高: 608.0
+最低: 593.0
+收盘: 605.0</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>• 毛利率：待更新
+• 净利率：約 11.0% (26Q2)
+• ROE：18.2% 年化 (26H1)
+• EPS：4.80 元 (26Q2)</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>2026Q2 已公告；下一次財報/法說日待公司公告</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>外资: +939 张
+投信: -802 张
+[2026-08-26 官方结算] 外资主力大幅回流 (+939 张)，投信阶段获利减仓 (-802 张)。</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>法人净买超 385 张 (占量 3.5%)
+[2026-08-26 筹码] 主力机构呈净买入 (+385 张)，筹码向法人端汇聚沉淀。</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>【Chokepoint 79分】卡位最上游铲子卖家，客户切换周期超 12-36 个月，垄断护城河极深。</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>NT$ 605.0</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>建议买点：小部位觀察
+黄金重仓：等待營益率連續改善</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>依封裝稼動率再評估</t>
+        </is>
+      </c>
+      <c r="M12" s="11" t="inlineStr">
+        <is>
+          <t>不預設固定目標</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr">
+        <is>
+          <t>資本支出與折舊失控即檢視</t>
+        </is>
+      </c>
+      <c r="O12" s="7" t="inlineStr">
+        <is>
+          <t>11,136 张</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="105" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>2454.TW</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>聯發科</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>高階 SoC、AI ASIC 設計/IP 與客戶軟硬體生態整合的高門檻</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>开盘: 4005.0
+最高: 4005.0
+最低: 3865.0
+收盘: 3865.0</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>• 毛利率：46.2% (26Q2)
+• 净利率：約 16.2% (26Q2)
+• ROE：待更新
+• EPS：15.28 元 (26Q2)</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>2026Q2 已公告；下一次財報/法說日待公司公告</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>外资: +1231 张
+投信: -227 张
+[2026-08-26 官方结算] 外资主力大幅回流 (+1,231 张)，投信阶段获利减仓 (-227 张)。</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>法人净买超 1,147 张 (占量 22.6%)
+[2026-08-26 筹码] 主力机构呈净买入 (+1,147 张)，筹码向法人端汇聚沉淀。</t>
+        </is>
+      </c>
+      <c r="I13" s="15" t="inlineStr">
+        <is>
+          <t>【Chokepoint 77分】卡位最上游铲子卖家，客户切换周期超 12-36 个月，垄断护城河极深。</t>
+        </is>
+      </c>
+      <c r="J13" s="17" t="inlineStr">
+        <is>
+          <t>NT$ 3865.0</t>
+        </is>
+      </c>
+      <c r="K13" s="18" t="inlineStr">
+        <is>
+          <t>建议买点：觀察，不追價
+黄金重仓：等待 AI ASIC 驗證</t>
+        </is>
+      </c>
+      <c r="L13" s="19" t="inlineStr">
+        <is>
+          <t>依 ASIC 營收再評估</t>
+        </is>
+      </c>
+      <c r="M13" s="20" t="inlineStr">
+        <is>
+          <t>不預設固定目標</t>
+        </is>
+      </c>
+      <c r="N13" s="21" t="inlineStr">
+        <is>
+          <t>獲利與 ASIC 時程轉弱即檢視</t>
+        </is>
+      </c>
+      <c r="O13" s="16" t="inlineStr">
+        <is>
+          <t>5,069 张</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1179,14 +1614,14 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>台股 5 大卡位龙头 Shioaji 实时买卖点与风控决策面板</t>
+          <t>台股 10 檔卡位龙头 Shioaji 实时买卖点与风控决策面板</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-08-26 15:24:17 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-08-27 16:29:12 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>
@@ -1250,22 +1685,22 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2375.0</t>
+          <t>NT$ 2430.0</t>
         </is>
       </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2425.0</t>
+          <t>NT$ 2435.0</t>
         </is>
       </c>
       <c r="E4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2375.0</t>
+          <t>NT$ 2410.0</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2415.0</t>
+          <t>NT$ 2410.0</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
@@ -1297,22 +1732,22 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 14295.0</t>
+          <t>NT$ 14695.0</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 14590.0</t>
+          <t>NT$ 14815.0</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 13855.0</t>
+          <t>NT$ 14085.0</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 14510.0</t>
+          <t>NT$ 14340.0</t>
         </is>
       </c>
       <c r="G5" s="29" t="inlineStr">
@@ -1344,22 +1779,22 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5565.0</t>
+          <t>NT$ 5960.0</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5920.0</t>
+          <t>NT$ 5960.0</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5555.0</t>
+          <t>NT$ 5355.0</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5895.0</t>
+          <t>NT$ 5500.0</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
@@ -1391,22 +1826,22 @@
       </c>
       <c r="C7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2880.0</t>
+          <t>NT$ 3305.0</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3155.0</t>
+          <t>NT$ 3440.0</t>
         </is>
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2850.0</t>
+          <t>NT$ 3265.0</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3155.0</t>
+          <t>NT$ 3340.0</t>
         </is>
       </c>
       <c r="G7" s="29" t="inlineStr">
@@ -1438,22 +1873,22 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 243.0</t>
+          <t>NT$ 248.5</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 248.0</t>
+          <t>NT$ 256.5</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 241.5</t>
+          <t>NT$ 248.5</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 246.5</t>
+          <t>NT$ 252.0</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
@@ -1469,6 +1904,241 @@
       <c r="I8" s="8" t="inlineStr">
         <is>
           <t>225 元</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>2308.TW</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>台達電</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 1780.0</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 1820.0</t>
+        </is>
+      </c>
+      <c r="E9" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 1760.0</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>NT$ 1770.0</t>
+        </is>
+      </c>
+      <c r="G9" s="29" t="inlineStr">
+        <is>
+          <t>分批觀察（不追高）</t>
+        </is>
+      </c>
+      <c r="H9" s="30" t="inlineStr">
+        <is>
+          <t>依獲利與趨勢再評估</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>跌破基本面假設即檢視</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2345.TW</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>智邦</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 2120.0</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 2130.0</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 2065.0</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>NT$ 2090.0</t>
+        </is>
+      </c>
+      <c r="G10" s="25" t="inlineStr">
+        <is>
+          <t>分批觀察（不追高）</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>依訂單與 EPS 趨勢再評估</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>營益率與訂單能見度轉弱即檢視</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>2360.TW</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>致茂</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 2010.0</t>
+        </is>
+      </c>
+      <c r="D11" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 2085.0</t>
+        </is>
+      </c>
+      <c r="E11" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 1970.0</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>NT$ 1990.0</t>
+        </is>
+      </c>
+      <c r="G11" s="29" t="inlineStr">
+        <is>
+          <t>回檔分批觀察</t>
+        </is>
+      </c>
+      <c r="H11" s="30" t="inlineStr">
+        <is>
+          <t>依 EPS 與毛利率再評估</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>獲利趨勢反轉即檢視</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>3711.TW</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>日月光投控</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 608.0</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 608.0</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 593.0</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>NT$ 605.0</t>
+        </is>
+      </c>
+      <c r="G12" s="25" t="inlineStr">
+        <is>
+          <t>小部位觀察</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>依封裝稼動率再評估</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>資本支出與折舊失控即檢視</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>2454.TW</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>聯發科</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 4005.0</t>
+        </is>
+      </c>
+      <c r="D13" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 4005.0</t>
+        </is>
+      </c>
+      <c r="E13" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 3865.0</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>NT$ 3865.0</t>
+        </is>
+      </c>
+      <c r="G13" s="29" t="inlineStr">
+        <is>
+          <t>觀察，不追價</t>
+        </is>
+      </c>
+      <c r="H13" s="30" t="inlineStr">
+        <is>
+          <t>依 ASIC 營收再評估</t>
+        </is>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>獲利與 ASIC 時程轉弱即檢視</t>
         </is>
       </c>
     </row>

</xml_diff>